<commit_message>
Saving data analysis just for fun
</commit_message>
<xml_diff>
--- a/DataAnalysis/LT/0.05/Results.xlsx
+++ b/DataAnalysis/LT/0.05/Results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Utente\Desktop\CultureAwarenessTest\DataAnalysis\LT\0.05\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FAD4F67-C8E8-49C7-B619-A51DC72E928D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{113FA43B-BBD4-47E3-9C49-BF3E5A6E1853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="77">
   <si>
     <t>Dati originali</t>
   </si>
@@ -681,8 +681,35 @@
       <c r="P3">
         <v>0.53575837561071948</v>
       </c>
-      <c r="R3" t="s">
-        <v>76</v>
+      <c r="R3">
+        <v>30.666666666666668</v>
+      </c>
+      <c r="S3">
+        <v>5.0579969684978323</v>
+      </c>
+      <c r="T3">
+        <v>30.666666666666668</v>
+      </c>
+      <c r="U3">
+        <v>4.5092497528228863</v>
+      </c>
+      <c r="V3">
+        <v>10.833333333333334</v>
+      </c>
+      <c r="W3">
+        <v>2.8431203515386652</v>
+      </c>
+      <c r="X3">
+        <v>24.055555555555557</v>
+      </c>
+      <c r="Y3">
+        <v>2.6943012562182544</v>
+      </c>
+      <c r="Z3">
+        <v>13.222222222222223</v>
+      </c>
+      <c r="AA3">
+        <v>4.3853713048590777</v>
       </c>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.3">
@@ -723,34 +750,34 @@
         <v>1.4174834246858978</v>
       </c>
       <c r="R4">
-        <v>29.5</v>
+        <v>31.7</v>
       </c>
       <c r="S4">
-        <v>4.9497474683058327</v>
+        <v>3.8013155617496484</v>
       </c>
       <c r="T4">
-        <v>28.25</v>
+        <v>30.7</v>
       </c>
       <c r="U4">
-        <v>6.0104076400856536</v>
+        <v>4.644889664997442</v>
       </c>
       <c r="V4">
-        <v>9.25</v>
+        <v>11.1</v>
       </c>
       <c r="W4">
-        <v>5.3033008588991066</v>
+        <v>3.3429029300893576</v>
       </c>
       <c r="X4">
-        <v>22.333333333333336</v>
+        <v>24.5</v>
       </c>
       <c r="Y4">
-        <v>5.4211519890968356</v>
+        <v>3.4176827757349777</v>
       </c>
       <c r="Z4">
-        <v>13.083333333333334</v>
+        <v>13.4</v>
       </c>
       <c r="AA4">
-        <v>0.11785113019775875</v>
+        <v>0.77817450199524985</v>
       </c>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.3">
@@ -1079,6 +1106,36 @@
       <c r="P20">
         <v>3.5207247329921398</v>
       </c>
+      <c r="R20">
+        <v>37.666666666666664</v>
+      </c>
+      <c r="S20">
+        <v>1.4433756729740643</v>
+      </c>
+      <c r="T20">
+        <v>33.333333333333336</v>
+      </c>
+      <c r="U20">
+        <v>4.5092497528228863</v>
+      </c>
+      <c r="V20">
+        <v>11.166666666666666</v>
+      </c>
+      <c r="W20">
+        <v>2.7537852736430528</v>
+      </c>
+      <c r="X20">
+        <v>27.388888888888886</v>
+      </c>
+      <c r="Y20">
+        <v>2.1430335024428788</v>
+      </c>
+      <c r="Z20">
+        <v>16.222222222222221</v>
+      </c>
+      <c r="AA20">
+        <v>2.6369876191790693</v>
+      </c>
     </row>
     <row r="21" spans="1:27" x14ac:dyDescent="0.3">
       <c r="C21" t="s">
@@ -1121,34 +1178,34 @@
         <v>76</v>
       </c>
       <c r="R21">
-        <v>27.25</v>
+        <v>26.625</v>
       </c>
       <c r="S21">
-        <v>2.4748737341529163</v>
+        <v>3.6371921404658658</v>
       </c>
       <c r="T21">
-        <v>25.75</v>
+        <v>27.625</v>
       </c>
       <c r="U21">
-        <v>0.35355339059327379</v>
+        <v>2.2126530078919591</v>
       </c>
       <c r="V21">
-        <v>9</v>
+        <v>8.5</v>
       </c>
       <c r="W21">
-        <v>0.70710678118654757</v>
+        <v>2.1602468994692869</v>
       </c>
       <c r="X21">
-        <v>20.6666666666667</v>
+        <v>20.916666666666668</v>
       </c>
       <c r="Y21">
-        <v>0.70710678118654757</v>
+        <v>1.707825127659933</v>
       </c>
       <c r="Z21">
-        <v>11.666666666666668</v>
+        <v>12.416666666666668</v>
       </c>
       <c r="AA21">
-        <v>1.4142135623730951</v>
+        <v>1.2583057392117916</v>
       </c>
     </row>
     <row r="22" spans="1:27" x14ac:dyDescent="0.3">
@@ -1339,6 +1396,36 @@
       </c>
       <c r="P30">
         <v>1.9254629073050034</v>
+      </c>
+      <c r="R30">
+        <v>22.333333333333332</v>
+      </c>
+      <c r="S30">
+        <v>3.2145502536643242</v>
+      </c>
+      <c r="T30">
+        <v>21</v>
+      </c>
+      <c r="U30">
+        <v>4</v>
+      </c>
+      <c r="V30">
+        <v>10.333333333333334</v>
+      </c>
+      <c r="W30">
+        <v>3.2532035493238571</v>
+      </c>
+      <c r="X30">
+        <v>17.888888888888889</v>
+      </c>
+      <c r="Y30">
+        <v>1.0584754935143132</v>
+      </c>
+      <c r="Z30">
+        <v>7.5555555555555562</v>
+      </c>
+      <c r="AA30">
+        <v>2.364866294865863</v>
       </c>
     </row>
     <row r="31" spans="1:27" x14ac:dyDescent="0.3">
@@ -1502,7 +1589,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25FCA91D-5E11-4BE7-9F8B-616A902FA88F}">
-  <dimension ref="A2:AF14"/>
+  <dimension ref="A2:AF16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="2" spans="1:32" x14ac:dyDescent="0.3">
@@ -2027,68 +2114,68 @@
         <v>90</v>
       </c>
       <c r="Q13">
-        <f t="shared" ref="Q10:Q14" si="6">AVERAGE(C13,D13)</f>
+        <f t="shared" ref="Q13:Q14" si="6">AVERAGE(C13,D13)</f>
         <v>25.5</v>
       </c>
       <c r="R13">
-        <f t="shared" ref="R10:R14" si="7">AVERAGE(H13,I13)</f>
+        <f t="shared" ref="R13:R14" si="7">AVERAGE(H13,I13)</f>
         <v>25.5</v>
       </c>
       <c r="S13">
-        <f t="shared" ref="S10:S14" si="8">AVERAGE(M13,N13)</f>
+        <f t="shared" ref="S13:S14" si="8">AVERAGE(M13,N13)</f>
         <v>9.5</v>
       </c>
       <c r="T13">
-        <f t="shared" ref="T10:T14" si="9">AVERAGE(Q13:S13)</f>
+        <f t="shared" ref="T13:T14" si="9">AVERAGE(Q13:S13)</f>
         <v>20.166666666666668</v>
       </c>
       <c r="U13">
         <f>AVERAGE(Q13:Q18)</f>
-        <v>27.25</v>
+        <v>26.625</v>
       </c>
       <c r="V13">
         <f>_xlfn.STDEV.S(Q13:Q18)</f>
-        <v>2.4748737341529163</v>
+        <v>3.6371921404658658</v>
       </c>
       <c r="W13">
         <f>AVERAGE(R13:R18)</f>
-        <v>25.75</v>
+        <v>27.625</v>
       </c>
       <c r="X13">
         <f>_xlfn.STDEV.S(R13:R18)</f>
-        <v>0.35355339059327379</v>
+        <v>2.2126530078919591</v>
       </c>
       <c r="Y13">
         <f>AVERAGE(S13:S18)</f>
-        <v>9</v>
+        <v>8.5</v>
       </c>
       <c r="Z13">
         <f>_xlfn.STDEV.S(S13:S18)</f>
-        <v>0.70710678118654757</v>
+        <v>2.1602468994692869</v>
       </c>
       <c r="AA13">
         <f>AVERAGE(T13:T18)</f>
-        <v>20.666666666666668</v>
+        <v>20.916666666666668</v>
       </c>
       <c r="AB13">
         <f>_xlfn.STDEV.S(T13:T18)</f>
-        <v>0.70710678118654757</v>
+        <v>1.707825127659933</v>
       </c>
       <c r="AC13">
-        <f t="shared" ref="AC10:AC14" si="10">MIN(Q13:S13)</f>
+        <f t="shared" ref="AC13:AC14" si="10">MIN(Q13:S13)</f>
         <v>9.5</v>
       </c>
       <c r="AD13">
-        <f t="shared" ref="AD10:AD14" si="11">T13-AC13</f>
+        <f t="shared" ref="AD13:AD14" si="11">T13-AC13</f>
         <v>10.666666666666668</v>
       </c>
       <c r="AE13">
         <f>AVERAGE(AD13:AD18)</f>
-        <v>11.666666666666668</v>
+        <v>12.416666666666668</v>
       </c>
       <c r="AF13">
         <f>_xlfn.STDEV.S(AD13:AD18)</f>
-        <v>1.4142135623730951</v>
+        <v>1.2583057392117916</v>
       </c>
     </row>
     <row r="14" spans="1:32" x14ac:dyDescent="0.3">
@@ -2150,6 +2237,130 @@
       </c>
       <c r="AD14">
         <f t="shared" si="11"/>
+        <v>12.666666666666668</v>
+      </c>
+    </row>
+    <row r="15" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B15">
+        <v>84</v>
+      </c>
+      <c r="C15">
+        <v>16</v>
+      </c>
+      <c r="D15">
+        <v>28</v>
+      </c>
+      <c r="E15">
+        <v>72</v>
+      </c>
+      <c r="G15">
+        <v>84</v>
+      </c>
+      <c r="H15">
+        <v>16</v>
+      </c>
+      <c r="I15">
+        <v>44</v>
+      </c>
+      <c r="J15">
+        <v>56</v>
+      </c>
+      <c r="L15">
+        <v>96</v>
+      </c>
+      <c r="M15">
+        <v>4</v>
+      </c>
+      <c r="N15">
+        <v>7</v>
+      </c>
+      <c r="O15">
+        <v>93</v>
+      </c>
+      <c r="Q15">
+        <f t="shared" ref="Q15:Q16" si="12">AVERAGE(C15,D15)</f>
+        <v>22</v>
+      </c>
+      <c r="R15">
+        <f t="shared" ref="R15:R16" si="13">AVERAGE(H15,I15)</f>
+        <v>30</v>
+      </c>
+      <c r="S15">
+        <f t="shared" ref="S15:S16" si="14">AVERAGE(M15,N15)</f>
+        <v>5.5</v>
+      </c>
+      <c r="T15">
+        <f t="shared" ref="T15:T16" si="15">AVERAGE(Q15:S15)</f>
+        <v>19.166666666666668</v>
+      </c>
+      <c r="AC15">
+        <f t="shared" ref="AC15:AC16" si="16">MIN(Q15:S15)</f>
+        <v>5.5</v>
+      </c>
+      <c r="AD15">
+        <f t="shared" ref="AD15:AD16" si="17">T15-AC15</f>
+        <v>13.666666666666668</v>
+      </c>
+    </row>
+    <row r="16" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B16">
+        <v>63</v>
+      </c>
+      <c r="C16">
+        <v>37</v>
+      </c>
+      <c r="D16">
+        <v>23</v>
+      </c>
+      <c r="E16">
+        <v>77</v>
+      </c>
+      <c r="G16">
+        <v>81</v>
+      </c>
+      <c r="H16">
+        <v>19</v>
+      </c>
+      <c r="I16">
+        <v>39</v>
+      </c>
+      <c r="J16">
+        <v>61</v>
+      </c>
+      <c r="L16">
+        <v>93</v>
+      </c>
+      <c r="M16">
+        <v>7</v>
+      </c>
+      <c r="N16">
+        <v>14</v>
+      </c>
+      <c r="O16">
+        <v>86</v>
+      </c>
+      <c r="Q16">
+        <f t="shared" si="12"/>
+        <v>30</v>
+      </c>
+      <c r="R16">
+        <f t="shared" si="13"/>
+        <v>29</v>
+      </c>
+      <c r="S16">
+        <f t="shared" si="14"/>
+        <v>10.5</v>
+      </c>
+      <c r="T16">
+        <f t="shared" si="15"/>
+        <v>23.166666666666668</v>
+      </c>
+      <c r="AC16">
+        <f t="shared" si="16"/>
+        <v>10.5</v>
+      </c>
+      <c r="AD16">
+        <f t="shared" si="17"/>
         <v>12.666666666666668</v>
       </c>
     </row>
@@ -2160,7 +2371,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8328B926-3ADF-46D7-8F68-CEFFC1D24F6E}">
-  <dimension ref="A2:AF10"/>
+  <dimension ref="A2:AF16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="2" spans="1:32" x14ac:dyDescent="0.3">
@@ -2699,6 +2910,232 @@
       <c r="AD10">
         <f t="shared" si="5"/>
         <v>14.666666666666668</v>
+      </c>
+    </row>
+    <row r="14" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B14">
+        <v>55</v>
+      </c>
+      <c r="C14">
+        <v>45</v>
+      </c>
+      <c r="D14">
+        <v>32</v>
+      </c>
+      <c r="E14">
+        <v>68</v>
+      </c>
+      <c r="G14">
+        <v>54</v>
+      </c>
+      <c r="H14">
+        <v>46</v>
+      </c>
+      <c r="I14">
+        <v>20</v>
+      </c>
+      <c r="J14">
+        <v>80</v>
+      </c>
+      <c r="L14">
+        <v>91</v>
+      </c>
+      <c r="M14">
+        <v>9</v>
+      </c>
+      <c r="N14">
+        <v>7</v>
+      </c>
+      <c r="O14">
+        <v>93</v>
+      </c>
+      <c r="Q14">
+        <f t="shared" ref="Q11:Q16" si="6">AVERAGE(C14,D14)</f>
+        <v>38.5</v>
+      </c>
+      <c r="R14">
+        <f t="shared" ref="R11:R16" si="7">AVERAGE(H14,I14)</f>
+        <v>33</v>
+      </c>
+      <c r="S14">
+        <f t="shared" ref="S11:S16" si="8">AVERAGE(M14,N14)</f>
+        <v>8</v>
+      </c>
+      <c r="T14">
+        <f t="shared" ref="T11:T16" si="9">AVERAGE(Q14:S14)</f>
+        <v>26.5</v>
+      </c>
+      <c r="U14">
+        <f>AVERAGE(Q14:Q20)</f>
+        <v>37.666666666666664</v>
+      </c>
+      <c r="V14">
+        <f>_xlfn.STDEV.S(Q14:Q20)</f>
+        <v>1.4433756729740643</v>
+      </c>
+      <c r="W14">
+        <f>AVERAGE(R14:R20)</f>
+        <v>33.333333333333336</v>
+      </c>
+      <c r="X14">
+        <f>_xlfn.STDEV.S(R14:R20)</f>
+        <v>4.5092497528228863</v>
+      </c>
+      <c r="Y14">
+        <f>AVERAGE(S14:S20)</f>
+        <v>11.166666666666666</v>
+      </c>
+      <c r="Z14">
+        <f>_xlfn.STDEV.S(S14:S20)</f>
+        <v>2.7537852736430528</v>
+      </c>
+      <c r="AA14">
+        <f>AVERAGE(T14:T20)</f>
+        <v>27.388888888888886</v>
+      </c>
+      <c r="AB14">
+        <f>_xlfn.STDEV.S(T14:T20)</f>
+        <v>2.1430335024428788</v>
+      </c>
+      <c r="AC14">
+        <f t="shared" ref="AC11:AC16" si="10">MIN(Q14:S14)</f>
+        <v>8</v>
+      </c>
+      <c r="AD14">
+        <f t="shared" ref="AD11:AD16" si="11">T14-AC14</f>
+        <v>18.5</v>
+      </c>
+      <c r="AE14">
+        <f>AVERAGE(AD14:AD20)</f>
+        <v>16.222222222222221</v>
+      </c>
+      <c r="AF14">
+        <f>_xlfn.STDEV.S(AD14:AD20)</f>
+        <v>2.6369876191790693</v>
+      </c>
+    </row>
+    <row r="15" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B15">
+        <v>54</v>
+      </c>
+      <c r="C15">
+        <v>46</v>
+      </c>
+      <c r="D15">
+        <v>26</v>
+      </c>
+      <c r="E15">
+        <v>74</v>
+      </c>
+      <c r="G15">
+        <v>71</v>
+      </c>
+      <c r="H15">
+        <v>29</v>
+      </c>
+      <c r="I15">
+        <v>29</v>
+      </c>
+      <c r="J15">
+        <v>71</v>
+      </c>
+      <c r="L15">
+        <v>88</v>
+      </c>
+      <c r="M15">
+        <v>12</v>
+      </c>
+      <c r="N15">
+        <v>13</v>
+      </c>
+      <c r="O15">
+        <v>87</v>
+      </c>
+      <c r="Q15">
+        <f t="shared" si="6"/>
+        <v>36</v>
+      </c>
+      <c r="R15">
+        <f t="shared" si="7"/>
+        <v>29</v>
+      </c>
+      <c r="S15">
+        <f t="shared" si="8"/>
+        <v>12.5</v>
+      </c>
+      <c r="T15">
+        <f t="shared" si="9"/>
+        <v>25.833333333333332</v>
+      </c>
+      <c r="AC15">
+        <f t="shared" si="10"/>
+        <v>12.5</v>
+      </c>
+      <c r="AD15">
+        <f t="shared" si="11"/>
+        <v>13.333333333333332</v>
+      </c>
+    </row>
+    <row r="16" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B16">
+        <v>43</v>
+      </c>
+      <c r="C16">
+        <v>57</v>
+      </c>
+      <c r="D16">
+        <v>20</v>
+      </c>
+      <c r="E16">
+        <v>80</v>
+      </c>
+      <c r="G16">
+        <v>48</v>
+      </c>
+      <c r="H16">
+        <v>52</v>
+      </c>
+      <c r="I16">
+        <v>24</v>
+      </c>
+      <c r="J16">
+        <v>76</v>
+      </c>
+      <c r="L16">
+        <v>90</v>
+      </c>
+      <c r="M16">
+        <v>10</v>
+      </c>
+      <c r="N16">
+        <v>16</v>
+      </c>
+      <c r="O16">
+        <v>84</v>
+      </c>
+      <c r="Q16">
+        <f t="shared" si="6"/>
+        <v>38.5</v>
+      </c>
+      <c r="R16">
+        <f t="shared" si="7"/>
+        <v>38</v>
+      </c>
+      <c r="S16">
+        <f t="shared" si="8"/>
+        <v>13</v>
+      </c>
+      <c r="T16">
+        <f t="shared" si="9"/>
+        <v>29.833333333333332</v>
+      </c>
+      <c r="AC16">
+        <f t="shared" si="10"/>
+        <v>13</v>
+      </c>
+      <c r="AD16">
+        <f t="shared" si="11"/>
+        <v>16.833333333333332</v>
       </c>
     </row>
   </sheetData>
@@ -8904,27 +9341,27 @@
       </c>
       <c r="AI12">
         <f>AVERAGE(Q16:Q24)</f>
-        <v>28.9</v>
+        <v>30.285714285714285</v>
       </c>
       <c r="AJ12">
         <f>_xlfn.STDEV.S(Q16:Q24)</f>
-        <v>4.1140004861448372</v>
+        <v>4.4050836433332261</v>
       </c>
       <c r="AK12">
         <f>AVERAGE(R16:R24)</f>
-        <v>29</v>
+        <v>29.5</v>
       </c>
       <c r="AL12">
         <f>_xlfn.STDEV.S(R16:R24)</f>
-        <v>3.9528470752104741</v>
+        <v>3.6968455021364721</v>
       </c>
       <c r="AM12">
         <f>AVERAGE(S16:S24)</f>
-        <v>9.8000000000000007</v>
+        <v>10.428571428571429</v>
       </c>
       <c r="AN12">
         <f>_xlfn.STDEV.S(S16:S24)</f>
-        <v>2.8853076092507024</v>
+        <v>2.7299049346783022</v>
       </c>
       <c r="AO12">
         <v>20.537037037037035</v>
@@ -9259,68 +9696,68 @@
         <v>92</v>
       </c>
       <c r="Q21">
-        <f t="shared" ref="Q19:Q22" si="6">AVERAGE(C21,D21)</f>
+        <f t="shared" ref="Q21:Q22" si="6">AVERAGE(C21,D21)</f>
         <v>26</v>
       </c>
       <c r="R21">
-        <f t="shared" ref="R19:R22" si="7">AVERAGE(H21:I21)</f>
+        <f t="shared" ref="R21:R22" si="7">AVERAGE(H21:I21)</f>
         <v>24</v>
       </c>
       <c r="S21">
-        <f t="shared" ref="S19:S22" si="8">AVERAGE(M21,N21)</f>
+        <f t="shared" ref="S21:S22" si="8">AVERAGE(M21,N21)</f>
         <v>5.5</v>
       </c>
       <c r="T21">
-        <f t="shared" ref="T19:T22" si="9">AVERAGE(Q21:S21)</f>
+        <f t="shared" ref="T21:T22" si="9">AVERAGE(Q21:S21)</f>
         <v>18.5</v>
       </c>
       <c r="U21">
-        <f t="shared" ref="U19:U22" si="10">MIN(Q21:S21)</f>
+        <f t="shared" ref="U21:U22" si="10">MIN(Q21:S21)</f>
         <v>5.5</v>
       </c>
       <c r="V21">
-        <f t="shared" ref="V19:V22" si="11">(T21-U21)</f>
+        <f t="shared" ref="V21:V22" si="11">(T21-U21)</f>
         <v>13</v>
       </c>
       <c r="W21">
-        <f>AVERAGE(Q21:Q23)</f>
-        <v>29.5</v>
+        <f>AVERAGE(Q21:Q25)</f>
+        <v>31.7</v>
       </c>
       <c r="X21">
-        <f>_xlfn.STDEV.S(Q21:Q23)</f>
-        <v>4.9497474683058327</v>
+        <f>_xlfn.STDEV.S(Q21:Q25)</f>
+        <v>3.8013155617496484</v>
       </c>
       <c r="Y21">
-        <f>AVERAGE(R21:R23)</f>
-        <v>28.25</v>
+        <f>AVERAGE(R21:R25)</f>
+        <v>30.7</v>
       </c>
       <c r="Z21">
-        <f>_xlfn.STDEV.S(R21:R23)</f>
-        <v>6.0104076400856536</v>
+        <f>_xlfn.STDEV.S(R21:R25)</f>
+        <v>4.644889664997442</v>
       </c>
       <c r="AA21">
-        <f>AVERAGE(S21:S23)</f>
-        <v>9.25</v>
+        <f>AVERAGE(S21:S25)</f>
+        <v>11.1</v>
       </c>
       <c r="AB21">
-        <f>_xlfn.STDEV.S(S21:S23)</f>
-        <v>5.3033008588991066</v>
+        <f>_xlfn.STDEV.S(S21:S25)</f>
+        <v>3.3429029300893576</v>
       </c>
       <c r="AC21">
-        <f>AVERAGE(T21:T23)</f>
-        <v>22.333333333333336</v>
+        <f>AVERAGE(T21:T25)</f>
+        <v>24.5</v>
       </c>
       <c r="AD21">
-        <f>_xlfn.STDEV.S(T21:T23)</f>
-        <v>5.4211519890968356</v>
+        <f>_xlfn.STDEV.S(T21:T25)</f>
+        <v>3.4176827757349777</v>
       </c>
       <c r="AE21">
-        <f>AVERAGE(V21:V23)</f>
-        <v>13.083333333333334</v>
+        <f>AVERAGE(V21:V25)</f>
+        <v>13.4</v>
       </c>
       <c r="AF21">
-        <f>_xlfn.STDEV.S(V21:V23)</f>
-        <v>0.11785113019775875</v>
+        <f>_xlfn.STDEV.S(V21:V25)</f>
+        <v>0.77817450199524985</v>
       </c>
     </row>
     <row r="22" spans="1:32" x14ac:dyDescent="0.3">
@@ -9385,6 +9822,192 @@
         <v>13.166666666666668</v>
       </c>
     </row>
+    <row r="23" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B23">
+        <v>57</v>
+      </c>
+      <c r="C23">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>30</v>
+      </c>
+      <c r="E23">
+        <v>70</v>
+      </c>
+      <c r="G23">
+        <v>79</v>
+      </c>
+      <c r="H23">
+        <v>21</v>
+      </c>
+      <c r="I23">
+        <v>35</v>
+      </c>
+      <c r="J23">
+        <v>65</v>
+      </c>
+      <c r="L23">
+        <v>94</v>
+      </c>
+      <c r="M23">
+        <v>6</v>
+      </c>
+      <c r="N23">
+        <v>21</v>
+      </c>
+      <c r="O23">
+        <v>79</v>
+      </c>
+      <c r="Q23">
+        <f t="shared" ref="Q23:Q25" si="12">AVERAGE(C23,D23)</f>
+        <v>36.5</v>
+      </c>
+      <c r="R23">
+        <f t="shared" ref="R23:R25" si="13">AVERAGE(H23:I23)</f>
+        <v>28</v>
+      </c>
+      <c r="S23">
+        <f t="shared" ref="S23:S25" si="14">AVERAGE(M23,N23)</f>
+        <v>13.5</v>
+      </c>
+      <c r="T23">
+        <f t="shared" ref="T23:T25" si="15">AVERAGE(Q23:S23)</f>
+        <v>26</v>
+      </c>
+      <c r="U23">
+        <f t="shared" ref="U23:U25" si="16">MIN(Q23:S23)</f>
+        <v>13.5</v>
+      </c>
+      <c r="V23">
+        <f t="shared" ref="V23:V25" si="17">(T23-U23)</f>
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B24">
+        <v>61</v>
+      </c>
+      <c r="C24">
+        <v>39</v>
+      </c>
+      <c r="D24">
+        <v>23</v>
+      </c>
+      <c r="E24">
+        <v>77</v>
+      </c>
+      <c r="G24">
+        <v>64</v>
+      </c>
+      <c r="H24">
+        <v>36</v>
+      </c>
+      <c r="I24">
+        <v>31</v>
+      </c>
+      <c r="J24">
+        <v>69</v>
+      </c>
+      <c r="L24">
+        <v>91</v>
+      </c>
+      <c r="M24">
+        <v>9</v>
+      </c>
+      <c r="N24">
+        <v>12</v>
+      </c>
+      <c r="O24">
+        <v>88</v>
+      </c>
+      <c r="Q24">
+        <f t="shared" si="12"/>
+        <v>31</v>
+      </c>
+      <c r="R24">
+        <f t="shared" si="13"/>
+        <v>33.5</v>
+      </c>
+      <c r="S24">
+        <f t="shared" si="14"/>
+        <v>10.5</v>
+      </c>
+      <c r="T24">
+        <f t="shared" si="15"/>
+        <v>25</v>
+      </c>
+      <c r="U24">
+        <f t="shared" si="16"/>
+        <v>10.5</v>
+      </c>
+      <c r="V24">
+        <f t="shared" si="17"/>
+        <v>14.5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B25">
+        <v>73</v>
+      </c>
+      <c r="C25">
+        <v>27</v>
+      </c>
+      <c r="D25">
+        <v>37</v>
+      </c>
+      <c r="E25">
+        <v>63</v>
+      </c>
+      <c r="G25">
+        <v>77</v>
+      </c>
+      <c r="H25">
+        <v>23</v>
+      </c>
+      <c r="I25">
+        <v>48</v>
+      </c>
+      <c r="J25">
+        <v>52</v>
+      </c>
+      <c r="L25">
+        <v>93</v>
+      </c>
+      <c r="M25">
+        <v>7</v>
+      </c>
+      <c r="N25">
+        <v>19</v>
+      </c>
+      <c r="O25">
+        <v>81</v>
+      </c>
+      <c r="Q25">
+        <f t="shared" si="12"/>
+        <v>32</v>
+      </c>
+      <c r="R25">
+        <f t="shared" si="13"/>
+        <v>35.5</v>
+      </c>
+      <c r="S25">
+        <f t="shared" si="14"/>
+        <v>13</v>
+      </c>
+      <c r="T25">
+        <f t="shared" si="15"/>
+        <v>26.833333333333332</v>
+      </c>
+      <c r="U25">
+        <f t="shared" si="16"/>
+        <v>13</v>
+      </c>
+      <c r="V25">
+        <f t="shared" si="17"/>
+        <v>13.833333333333332</v>
+      </c>
+    </row>
     <row r="26" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>26</v>
@@ -10245,53 +10868,53 @@
     </row>
     <row r="68" spans="1:32" x14ac:dyDescent="0.3">
       <c r="Q68" t="e">
-        <f t="shared" ref="Q68:Q109" si="12">AVERAGE(C68,D68)</f>
+        <f t="shared" ref="Q68:Q109" si="18">AVERAGE(C68,D68)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="R68" t="e">
-        <f t="shared" ref="R68:R109" si="13">AVERAGE(H68:I68)</f>
+        <f t="shared" ref="R68:R109" si="19">AVERAGE(H68:I68)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="S68" t="e">
-        <f t="shared" ref="S68:S109" si="14">AVERAGE(M68,N68)</f>
+        <f t="shared" ref="S68:S109" si="20">AVERAGE(M68,N68)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="T68" t="e">
-        <f t="shared" ref="T68:T109" si="15">AVERAGE(Q68:S68)</f>
+        <f t="shared" ref="T68:T109" si="21">AVERAGE(Q68:S68)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="U68" t="e">
-        <f t="shared" ref="U68:U109" si="16">MIN(Q68:S68)</f>
+        <f t="shared" ref="U68:U109" si="22">MIN(Q68:S68)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="V68" t="e">
-        <f t="shared" ref="V68:V109" si="17">(1/3)*(T68-U68)</f>
+        <f t="shared" ref="V68:V109" si="23">(1/3)*(T68-U68)</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="69" spans="1:32" x14ac:dyDescent="0.3">
       <c r="Q69" t="e">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>#DIV/0!</v>
       </c>
       <c r="R69" t="e">
-        <f t="shared" si="13"/>
+        <f t="shared" si="19"/>
         <v>#DIV/0!</v>
       </c>
       <c r="S69" t="e">
-        <f t="shared" si="14"/>
+        <f t="shared" si="20"/>
         <v>#DIV/0!</v>
       </c>
       <c r="T69" t="e">
-        <f t="shared" si="15"/>
+        <f t="shared" si="21"/>
         <v>#DIV/0!</v>
       </c>
       <c r="U69" t="e">
-        <f t="shared" si="16"/>
+        <f t="shared" si="22"/>
         <v>#DIV/0!</v>
       </c>
       <c r="V69" t="e">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -10307,27 +10930,27 @@
     </row>
     <row r="73" spans="1:32" x14ac:dyDescent="0.3">
       <c r="Q73" t="e">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>#DIV/0!</v>
       </c>
       <c r="R73" t="e">
-        <f t="shared" si="13"/>
+        <f t="shared" si="19"/>
         <v>#DIV/0!</v>
       </c>
       <c r="S73" t="e">
-        <f t="shared" si="14"/>
+        <f t="shared" si="20"/>
         <v>#DIV/0!</v>
       </c>
       <c r="T73" t="e">
-        <f t="shared" si="15"/>
+        <f t="shared" si="21"/>
         <v>#DIV/0!</v>
       </c>
       <c r="U73" t="e">
-        <f t="shared" si="16"/>
+        <f t="shared" si="22"/>
         <v>#DIV/0!</v>
       </c>
       <c r="V73" t="e">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v>#DIV/0!</v>
       </c>
       <c r="AC73" t="e">
@@ -10349,53 +10972,53 @@
     </row>
     <row r="74" spans="1:32" x14ac:dyDescent="0.3">
       <c r="Q74" t="e">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>#DIV/0!</v>
       </c>
       <c r="R74" t="e">
-        <f t="shared" si="13"/>
+        <f t="shared" si="19"/>
         <v>#DIV/0!</v>
       </c>
       <c r="S74" t="e">
-        <f t="shared" si="14"/>
+        <f t="shared" si="20"/>
         <v>#DIV/0!</v>
       </c>
       <c r="T74" t="e">
-        <f t="shared" si="15"/>
+        <f t="shared" si="21"/>
         <v>#DIV/0!</v>
       </c>
       <c r="U74" t="e">
-        <f t="shared" si="16"/>
+        <f t="shared" si="22"/>
         <v>#DIV/0!</v>
       </c>
       <c r="V74" t="e">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="75" spans="1:32" x14ac:dyDescent="0.3">
       <c r="Q75" t="e">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>#DIV/0!</v>
       </c>
       <c r="R75" t="e">
-        <f t="shared" si="13"/>
+        <f t="shared" si="19"/>
         <v>#DIV/0!</v>
       </c>
       <c r="S75" t="e">
-        <f t="shared" si="14"/>
+        <f t="shared" si="20"/>
         <v>#DIV/0!</v>
       </c>
       <c r="T75" t="e">
-        <f t="shared" si="15"/>
+        <f t="shared" si="21"/>
         <v>#DIV/0!</v>
       </c>
       <c r="U75" t="e">
-        <f t="shared" si="16"/>
+        <f t="shared" si="22"/>
         <v>#DIV/0!</v>
       </c>
       <c r="V75" t="e">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -10411,27 +11034,27 @@
     </row>
     <row r="79" spans="1:32" x14ac:dyDescent="0.3">
       <c r="Q79" t="e">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>#DIV/0!</v>
       </c>
       <c r="R79" t="e">
-        <f t="shared" si="13"/>
+        <f t="shared" si="19"/>
         <v>#DIV/0!</v>
       </c>
       <c r="S79" t="e">
-        <f t="shared" si="14"/>
+        <f t="shared" si="20"/>
         <v>#DIV/0!</v>
       </c>
       <c r="T79" t="e">
-        <f t="shared" si="15"/>
+        <f t="shared" si="21"/>
         <v>#DIV/0!</v>
       </c>
       <c r="U79" t="e">
-        <f t="shared" si="16"/>
+        <f t="shared" si="22"/>
         <v>#DIV/0!</v>
       </c>
       <c r="V79" t="e">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v>#DIV/0!</v>
       </c>
       <c r="AC79" t="e">
@@ -10453,235 +11076,235 @@
     </row>
     <row r="80" spans="1:32" x14ac:dyDescent="0.3">
       <c r="Q80" t="e">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>#DIV/0!</v>
       </c>
       <c r="R80" t="e">
-        <f t="shared" si="13"/>
+        <f t="shared" si="19"/>
         <v>#DIV/0!</v>
       </c>
       <c r="S80" t="e">
-        <f t="shared" si="14"/>
+        <f t="shared" si="20"/>
         <v>#DIV/0!</v>
       </c>
       <c r="T80" t="e">
-        <f t="shared" si="15"/>
+        <f t="shared" si="21"/>
         <v>#DIV/0!</v>
       </c>
       <c r="U80" t="e">
-        <f t="shared" si="16"/>
+        <f t="shared" si="22"/>
         <v>#DIV/0!</v>
       </c>
       <c r="V80" t="e">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="81" spans="1:32" x14ac:dyDescent="0.3">
       <c r="Q81" t="e">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>#DIV/0!</v>
       </c>
       <c r="R81" t="e">
-        <f t="shared" si="13"/>
+        <f t="shared" si="19"/>
         <v>#DIV/0!</v>
       </c>
       <c r="S81" t="e">
-        <f t="shared" si="14"/>
+        <f t="shared" si="20"/>
         <v>#DIV/0!</v>
       </c>
       <c r="T81" t="e">
-        <f t="shared" si="15"/>
+        <f t="shared" si="21"/>
         <v>#DIV/0!</v>
       </c>
       <c r="U81" t="e">
-        <f t="shared" si="16"/>
+        <f t="shared" si="22"/>
         <v>#DIV/0!</v>
       </c>
       <c r="V81" t="e">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="82" spans="1:32" x14ac:dyDescent="0.3">
       <c r="Q82" t="e">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>#DIV/0!</v>
       </c>
       <c r="R82" t="e">
-        <f t="shared" si="13"/>
+        <f t="shared" si="19"/>
         <v>#DIV/0!</v>
       </c>
       <c r="S82" t="e">
-        <f t="shared" si="14"/>
+        <f t="shared" si="20"/>
         <v>#DIV/0!</v>
       </c>
       <c r="T82" t="e">
-        <f t="shared" si="15"/>
+        <f t="shared" si="21"/>
         <v>#DIV/0!</v>
       </c>
       <c r="U82" t="e">
-        <f t="shared" si="16"/>
+        <f t="shared" si="22"/>
         <v>#DIV/0!</v>
       </c>
       <c r="V82" t="e">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="83" spans="1:32" x14ac:dyDescent="0.3">
       <c r="Q83" t="e">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>#DIV/0!</v>
       </c>
       <c r="R83" t="e">
-        <f t="shared" si="13"/>
+        <f t="shared" si="19"/>
         <v>#DIV/0!</v>
       </c>
       <c r="S83" t="e">
-        <f t="shared" si="14"/>
+        <f t="shared" si="20"/>
         <v>#DIV/0!</v>
       </c>
       <c r="T83" t="e">
-        <f t="shared" si="15"/>
+        <f t="shared" si="21"/>
         <v>#DIV/0!</v>
       </c>
       <c r="U83" t="e">
-        <f t="shared" si="16"/>
+        <f t="shared" si="22"/>
         <v>#DIV/0!</v>
       </c>
       <c r="V83" t="e">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="84" spans="1:32" x14ac:dyDescent="0.3">
       <c r="Q84" t="e">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>#DIV/0!</v>
       </c>
       <c r="R84" t="e">
-        <f t="shared" si="13"/>
+        <f t="shared" si="19"/>
         <v>#DIV/0!</v>
       </c>
       <c r="S84" t="e">
-        <f t="shared" si="14"/>
+        <f t="shared" si="20"/>
         <v>#DIV/0!</v>
       </c>
       <c r="T84" t="e">
-        <f t="shared" si="15"/>
+        <f t="shared" si="21"/>
         <v>#DIV/0!</v>
       </c>
       <c r="U84" t="e">
-        <f t="shared" si="16"/>
+        <f t="shared" si="22"/>
         <v>#DIV/0!</v>
       </c>
       <c r="V84" t="e">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="85" spans="1:32" x14ac:dyDescent="0.3">
       <c r="Q85" t="e">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>#DIV/0!</v>
       </c>
       <c r="R85" t="e">
-        <f t="shared" si="13"/>
+        <f t="shared" si="19"/>
         <v>#DIV/0!</v>
       </c>
       <c r="S85" t="e">
-        <f t="shared" si="14"/>
+        <f t="shared" si="20"/>
         <v>#DIV/0!</v>
       </c>
       <c r="T85" t="e">
-        <f t="shared" si="15"/>
+        <f t="shared" si="21"/>
         <v>#DIV/0!</v>
       </c>
       <c r="U85" t="e">
-        <f t="shared" si="16"/>
+        <f t="shared" si="22"/>
         <v>#DIV/0!</v>
       </c>
       <c r="V85" t="e">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="86" spans="1:32" x14ac:dyDescent="0.3">
       <c r="Q86" t="e">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>#DIV/0!</v>
       </c>
       <c r="R86" t="e">
-        <f t="shared" si="13"/>
+        <f t="shared" si="19"/>
         <v>#DIV/0!</v>
       </c>
       <c r="S86" t="e">
-        <f t="shared" si="14"/>
+        <f t="shared" si="20"/>
         <v>#DIV/0!</v>
       </c>
       <c r="T86" t="e">
-        <f t="shared" si="15"/>
+        <f t="shared" si="21"/>
         <v>#DIV/0!</v>
       </c>
       <c r="U86" t="e">
-        <f t="shared" si="16"/>
+        <f t="shared" si="22"/>
         <v>#DIV/0!</v>
       </c>
       <c r="V86" t="e">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="87" spans="1:32" x14ac:dyDescent="0.3">
       <c r="Q87" t="e">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>#DIV/0!</v>
       </c>
       <c r="R87" t="e">
-        <f t="shared" si="13"/>
+        <f t="shared" si="19"/>
         <v>#DIV/0!</v>
       </c>
       <c r="S87" t="e">
-        <f t="shared" si="14"/>
+        <f t="shared" si="20"/>
         <v>#DIV/0!</v>
       </c>
       <c r="T87" t="e">
-        <f t="shared" si="15"/>
+        <f t="shared" si="21"/>
         <v>#DIV/0!</v>
       </c>
       <c r="U87" t="e">
-        <f t="shared" si="16"/>
+        <f t="shared" si="22"/>
         <v>#DIV/0!</v>
       </c>
       <c r="V87" t="e">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="88" spans="1:32" x14ac:dyDescent="0.3">
       <c r="Q88" t="e">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>#DIV/0!</v>
       </c>
       <c r="R88" t="e">
-        <f t="shared" si="13"/>
+        <f t="shared" si="19"/>
         <v>#DIV/0!</v>
       </c>
       <c r="S88" t="e">
-        <f t="shared" si="14"/>
+        <f t="shared" si="20"/>
         <v>#DIV/0!</v>
       </c>
       <c r="T88" t="e">
-        <f t="shared" si="15"/>
+        <f t="shared" si="21"/>
         <v>#DIV/0!</v>
       </c>
       <c r="U88" t="e">
-        <f t="shared" si="16"/>
+        <f t="shared" si="22"/>
         <v>#DIV/0!</v>
       </c>
       <c r="V88" t="e">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -10697,27 +11320,27 @@
     </row>
     <row r="92" spans="1:32" x14ac:dyDescent="0.3">
       <c r="Q92" t="e">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>#DIV/0!</v>
       </c>
       <c r="R92" t="e">
-        <f t="shared" si="13"/>
+        <f t="shared" si="19"/>
         <v>#DIV/0!</v>
       </c>
       <c r="S92" t="e">
-        <f t="shared" si="14"/>
+        <f t="shared" si="20"/>
         <v>#DIV/0!</v>
       </c>
       <c r="T92" t="e">
-        <f t="shared" si="15"/>
+        <f t="shared" si="21"/>
         <v>#DIV/0!</v>
       </c>
       <c r="U92" t="e">
-        <f t="shared" si="16"/>
+        <f t="shared" si="22"/>
         <v>#DIV/0!</v>
       </c>
       <c r="V92" t="e">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v>#DIV/0!</v>
       </c>
       <c r="AC92" t="e">
@@ -10739,131 +11362,131 @@
     </row>
     <row r="93" spans="1:32" x14ac:dyDescent="0.3">
       <c r="Q93" t="e">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>#DIV/0!</v>
       </c>
       <c r="R93" t="e">
-        <f t="shared" si="13"/>
+        <f t="shared" si="19"/>
         <v>#DIV/0!</v>
       </c>
       <c r="S93" t="e">
-        <f t="shared" si="14"/>
+        <f t="shared" si="20"/>
         <v>#DIV/0!</v>
       </c>
       <c r="T93" t="e">
-        <f t="shared" si="15"/>
+        <f t="shared" si="21"/>
         <v>#DIV/0!</v>
       </c>
       <c r="U93" t="e">
-        <f t="shared" si="16"/>
+        <f t="shared" si="22"/>
         <v>#DIV/0!</v>
       </c>
       <c r="V93" t="e">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="94" spans="1:32" x14ac:dyDescent="0.3">
       <c r="Q94" t="e">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>#DIV/0!</v>
       </c>
       <c r="R94" t="e">
-        <f t="shared" si="13"/>
+        <f t="shared" si="19"/>
         <v>#DIV/0!</v>
       </c>
       <c r="S94" t="e">
-        <f t="shared" si="14"/>
+        <f t="shared" si="20"/>
         <v>#DIV/0!</v>
       </c>
       <c r="T94" t="e">
-        <f t="shared" si="15"/>
+        <f t="shared" si="21"/>
         <v>#DIV/0!</v>
       </c>
       <c r="U94" t="e">
-        <f t="shared" si="16"/>
+        <f t="shared" si="22"/>
         <v>#DIV/0!</v>
       </c>
       <c r="V94" t="e">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="95" spans="1:32" x14ac:dyDescent="0.3">
       <c r="Q95" t="e">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>#DIV/0!</v>
       </c>
       <c r="R95" t="e">
-        <f t="shared" si="13"/>
+        <f t="shared" si="19"/>
         <v>#DIV/0!</v>
       </c>
       <c r="S95" t="e">
-        <f t="shared" si="14"/>
+        <f t="shared" si="20"/>
         <v>#DIV/0!</v>
       </c>
       <c r="T95" t="e">
-        <f t="shared" si="15"/>
+        <f t="shared" si="21"/>
         <v>#DIV/0!</v>
       </c>
       <c r="U95" t="e">
-        <f t="shared" si="16"/>
+        <f t="shared" si="22"/>
         <v>#DIV/0!</v>
       </c>
       <c r="V95" t="e">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="96" spans="1:32" x14ac:dyDescent="0.3">
       <c r="Q96" t="e">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>#DIV/0!</v>
       </c>
       <c r="R96" t="e">
-        <f t="shared" si="13"/>
+        <f t="shared" si="19"/>
         <v>#DIV/0!</v>
       </c>
       <c r="S96" t="e">
-        <f t="shared" si="14"/>
+        <f t="shared" si="20"/>
         <v>#DIV/0!</v>
       </c>
       <c r="T96" t="e">
-        <f t="shared" si="15"/>
+        <f t="shared" si="21"/>
         <v>#DIV/0!</v>
       </c>
       <c r="U96" t="e">
-        <f t="shared" si="16"/>
+        <f t="shared" si="22"/>
         <v>#DIV/0!</v>
       </c>
       <c r="V96" t="e">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="97" spans="1:32" x14ac:dyDescent="0.3">
       <c r="Q97" t="e">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>#DIV/0!</v>
       </c>
       <c r="R97" t="e">
-        <f t="shared" si="13"/>
+        <f t="shared" si="19"/>
         <v>#DIV/0!</v>
       </c>
       <c r="S97" t="e">
-        <f t="shared" si="14"/>
+        <f t="shared" si="20"/>
         <v>#DIV/0!</v>
       </c>
       <c r="T97" t="e">
-        <f t="shared" si="15"/>
+        <f t="shared" si="21"/>
         <v>#DIV/0!</v>
       </c>
       <c r="U97" t="e">
-        <f t="shared" si="16"/>
+        <f t="shared" si="22"/>
         <v>#DIV/0!</v>
       </c>
       <c r="V97" t="e">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -10879,27 +11502,27 @@
     </row>
     <row r="101" spans="1:32" x14ac:dyDescent="0.3">
       <c r="Q101" t="e">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>#DIV/0!</v>
       </c>
       <c r="R101" t="e">
-        <f t="shared" si="13"/>
+        <f t="shared" si="19"/>
         <v>#DIV/0!</v>
       </c>
       <c r="S101" t="e">
-        <f t="shared" si="14"/>
+        <f t="shared" si="20"/>
         <v>#DIV/0!</v>
       </c>
       <c r="T101" t="e">
-        <f t="shared" si="15"/>
+        <f t="shared" si="21"/>
         <v>#DIV/0!</v>
       </c>
       <c r="U101" t="e">
-        <f t="shared" si="16"/>
+        <f t="shared" si="22"/>
         <v>#DIV/0!</v>
       </c>
       <c r="V101" t="e">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v>#DIV/0!</v>
       </c>
       <c r="AC101" t="e">
@@ -10921,209 +11544,209 @@
     </row>
     <row r="102" spans="1:32" x14ac:dyDescent="0.3">
       <c r="Q102" t="e">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>#DIV/0!</v>
       </c>
       <c r="R102" t="e">
-        <f t="shared" si="13"/>
+        <f t="shared" si="19"/>
         <v>#DIV/0!</v>
       </c>
       <c r="S102" t="e">
-        <f t="shared" si="14"/>
+        <f t="shared" si="20"/>
         <v>#DIV/0!</v>
       </c>
       <c r="T102" t="e">
-        <f t="shared" si="15"/>
+        <f t="shared" si="21"/>
         <v>#DIV/0!</v>
       </c>
       <c r="U102" t="e">
-        <f t="shared" si="16"/>
+        <f t="shared" si="22"/>
         <v>#DIV/0!</v>
       </c>
       <c r="V102" t="e">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="103" spans="1:32" x14ac:dyDescent="0.3">
       <c r="Q103" t="e">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>#DIV/0!</v>
       </c>
       <c r="R103" t="e">
-        <f t="shared" si="13"/>
+        <f t="shared" si="19"/>
         <v>#DIV/0!</v>
       </c>
       <c r="S103" t="e">
-        <f t="shared" si="14"/>
+        <f t="shared" si="20"/>
         <v>#DIV/0!</v>
       </c>
       <c r="T103" t="e">
-        <f t="shared" si="15"/>
+        <f t="shared" si="21"/>
         <v>#DIV/0!</v>
       </c>
       <c r="U103" t="e">
-        <f t="shared" si="16"/>
+        <f t="shared" si="22"/>
         <v>#DIV/0!</v>
       </c>
       <c r="V103" t="e">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="104" spans="1:32" x14ac:dyDescent="0.3">
       <c r="Q104" t="e">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>#DIV/0!</v>
       </c>
       <c r="R104" t="e">
-        <f t="shared" si="13"/>
+        <f t="shared" si="19"/>
         <v>#DIV/0!</v>
       </c>
       <c r="S104" t="e">
-        <f t="shared" si="14"/>
+        <f t="shared" si="20"/>
         <v>#DIV/0!</v>
       </c>
       <c r="T104" t="e">
-        <f t="shared" si="15"/>
+        <f t="shared" si="21"/>
         <v>#DIV/0!</v>
       </c>
       <c r="U104" t="e">
-        <f t="shared" si="16"/>
+        <f t="shared" si="22"/>
         <v>#DIV/0!</v>
       </c>
       <c r="V104" t="e">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="105" spans="1:32" x14ac:dyDescent="0.3">
       <c r="Q105" t="e">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>#DIV/0!</v>
       </c>
       <c r="R105" t="e">
-        <f t="shared" si="13"/>
+        <f t="shared" si="19"/>
         <v>#DIV/0!</v>
       </c>
       <c r="S105" t="e">
-        <f t="shared" si="14"/>
+        <f t="shared" si="20"/>
         <v>#DIV/0!</v>
       </c>
       <c r="T105" t="e">
-        <f t="shared" si="15"/>
+        <f t="shared" si="21"/>
         <v>#DIV/0!</v>
       </c>
       <c r="U105" t="e">
-        <f t="shared" si="16"/>
+        <f t="shared" si="22"/>
         <v>#DIV/0!</v>
       </c>
       <c r="V105" t="e">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="106" spans="1:32" x14ac:dyDescent="0.3">
       <c r="Q106" t="e">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>#DIV/0!</v>
       </c>
       <c r="R106" t="e">
-        <f t="shared" si="13"/>
+        <f t="shared" si="19"/>
         <v>#DIV/0!</v>
       </c>
       <c r="S106" t="e">
-        <f t="shared" si="14"/>
+        <f t="shared" si="20"/>
         <v>#DIV/0!</v>
       </c>
       <c r="T106" t="e">
-        <f t="shared" si="15"/>
+        <f t="shared" si="21"/>
         <v>#DIV/0!</v>
       </c>
       <c r="U106" t="e">
-        <f t="shared" si="16"/>
+        <f t="shared" si="22"/>
         <v>#DIV/0!</v>
       </c>
       <c r="V106" t="e">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="107" spans="1:32" x14ac:dyDescent="0.3">
       <c r="Q107" t="e">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>#DIV/0!</v>
       </c>
       <c r="R107" t="e">
-        <f t="shared" si="13"/>
+        <f t="shared" si="19"/>
         <v>#DIV/0!</v>
       </c>
       <c r="S107" t="e">
-        <f t="shared" si="14"/>
+        <f t="shared" si="20"/>
         <v>#DIV/0!</v>
       </c>
       <c r="T107" t="e">
-        <f t="shared" si="15"/>
+        <f t="shared" si="21"/>
         <v>#DIV/0!</v>
       </c>
       <c r="U107" t="e">
-        <f t="shared" si="16"/>
+        <f t="shared" si="22"/>
         <v>#DIV/0!</v>
       </c>
       <c r="V107" t="e">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="108" spans="1:32" x14ac:dyDescent="0.3">
       <c r="Q108" t="e">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>#DIV/0!</v>
       </c>
       <c r="R108" t="e">
-        <f t="shared" si="13"/>
+        <f t="shared" si="19"/>
         <v>#DIV/0!</v>
       </c>
       <c r="S108" t="e">
-        <f t="shared" si="14"/>
+        <f t="shared" si="20"/>
         <v>#DIV/0!</v>
       </c>
       <c r="T108" t="e">
-        <f t="shared" si="15"/>
+        <f t="shared" si="21"/>
         <v>#DIV/0!</v>
       </c>
       <c r="U108" t="e">
-        <f t="shared" si="16"/>
+        <f t="shared" si="22"/>
         <v>#DIV/0!</v>
       </c>
       <c r="V108" t="e">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="109" spans="1:32" x14ac:dyDescent="0.3">
       <c r="Q109" t="e">
-        <f t="shared" si="12"/>
+        <f t="shared" si="18"/>
         <v>#DIV/0!</v>
       </c>
       <c r="R109" t="e">
-        <f t="shared" si="13"/>
+        <f t="shared" si="19"/>
         <v>#DIV/0!</v>
       </c>
       <c r="S109" t="e">
-        <f t="shared" si="14"/>
+        <f t="shared" si="20"/>
         <v>#DIV/0!</v>
       </c>
       <c r="T109" t="e">
-        <f t="shared" si="15"/>
+        <f t="shared" si="21"/>
         <v>#DIV/0!</v>
       </c>
       <c r="U109" t="e">
-        <f t="shared" si="16"/>
+        <f t="shared" si="22"/>
         <v>#DIV/0!</v>
       </c>
       <c r="V109" t="e">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -11134,7 +11757,7 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D80BAE23-A740-4698-B840-F018E78CD098}">
-  <dimension ref="A1:AF5"/>
+  <dimension ref="A1:AF11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="23" max="23" width="13.109375" customWidth="1"/>
@@ -11425,6 +12048,232 @@
       <c r="V5">
         <f t="shared" si="5"/>
         <v>14.833333333333332</v>
+      </c>
+    </row>
+    <row r="9" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B9">
+        <v>64</v>
+      </c>
+      <c r="C9">
+        <v>36</v>
+      </c>
+      <c r="D9">
+        <v>20</v>
+      </c>
+      <c r="E9">
+        <v>80</v>
+      </c>
+      <c r="G9">
+        <v>72</v>
+      </c>
+      <c r="H9">
+        <v>28</v>
+      </c>
+      <c r="I9">
+        <v>34</v>
+      </c>
+      <c r="J9">
+        <v>66</v>
+      </c>
+      <c r="L9">
+        <v>92</v>
+      </c>
+      <c r="M9">
+        <v>8</v>
+      </c>
+      <c r="N9">
+        <v>9</v>
+      </c>
+      <c r="O9">
+        <v>91</v>
+      </c>
+      <c r="Q9">
+        <f t="shared" ref="Q6:Q11" si="6">AVERAGE(C9:D9)</f>
+        <v>28</v>
+      </c>
+      <c r="R9">
+        <f t="shared" ref="R6:R11" si="7">AVERAGE(H9:I9)</f>
+        <v>31</v>
+      </c>
+      <c r="S9">
+        <f t="shared" ref="S6:S11" si="8">AVERAGE(M9:N9)</f>
+        <v>8.5</v>
+      </c>
+      <c r="T9">
+        <f t="shared" ref="T6:T11" si="9">AVERAGE(Q9:S9)</f>
+        <v>22.5</v>
+      </c>
+      <c r="U9">
+        <f t="shared" ref="U6:U11" si="10">MIN(Q9:S9)</f>
+        <v>8.5</v>
+      </c>
+      <c r="V9">
+        <f t="shared" ref="V6:V11" si="11">T9-U9</f>
+        <v>14</v>
+      </c>
+      <c r="W9">
+        <f>AVERAGE(Q9:Q11)</f>
+        <v>30.666666666666668</v>
+      </c>
+      <c r="X9">
+        <f>_xlfn.STDEV.S(Q9:Q11)</f>
+        <v>5.0579969684978323</v>
+      </c>
+      <c r="Y9">
+        <f>AVERAGE(R9:R11)</f>
+        <v>30.666666666666668</v>
+      </c>
+      <c r="Z9">
+        <f>_xlfn.STDEV.S(R9:R11)</f>
+        <v>4.5092497528228863</v>
+      </c>
+      <c r="AA9">
+        <f>AVERAGE(S9:S11)</f>
+        <v>10.833333333333334</v>
+      </c>
+      <c r="AB9">
+        <f>_xlfn.STDEV.S(S9:S11)</f>
+        <v>2.8431203515386652</v>
+      </c>
+      <c r="AC9">
+        <f>AVERAGE(T9:T11)</f>
+        <v>24.055555555555557</v>
+      </c>
+      <c r="AD9">
+        <f>_xlfn.STDEV.S(T9:T11)</f>
+        <v>2.6943012562182544</v>
+      </c>
+      <c r="AE9">
+        <f>AVERAGE(V9:V11)</f>
+        <v>13.222222222222223</v>
+      </c>
+      <c r="AF9">
+        <f>_xlfn.STDEV.S(V9:V11)</f>
+        <v>4.3853713048590777</v>
+      </c>
+    </row>
+    <row r="10" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B10">
+        <v>71</v>
+      </c>
+      <c r="C10">
+        <v>29</v>
+      </c>
+      <c r="D10">
+        <v>26</v>
+      </c>
+      <c r="E10">
+        <v>74</v>
+      </c>
+      <c r="G10">
+        <v>72</v>
+      </c>
+      <c r="H10">
+        <v>28</v>
+      </c>
+      <c r="I10">
+        <v>24</v>
+      </c>
+      <c r="J10">
+        <v>76</v>
+      </c>
+      <c r="L10">
+        <v>89</v>
+      </c>
+      <c r="M10">
+        <v>11</v>
+      </c>
+      <c r="N10">
+        <v>17</v>
+      </c>
+      <c r="O10">
+        <v>83</v>
+      </c>
+      <c r="Q10">
+        <f t="shared" si="6"/>
+        <v>27.5</v>
+      </c>
+      <c r="R10">
+        <f t="shared" si="7"/>
+        <v>26</v>
+      </c>
+      <c r="S10">
+        <f t="shared" si="8"/>
+        <v>14</v>
+      </c>
+      <c r="T10">
+        <f t="shared" si="9"/>
+        <v>22.5</v>
+      </c>
+      <c r="U10">
+        <f t="shared" si="10"/>
+        <v>14</v>
+      </c>
+      <c r="V10">
+        <f t="shared" si="11"/>
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B11">
+        <v>53</v>
+      </c>
+      <c r="C11">
+        <v>47</v>
+      </c>
+      <c r="D11">
+        <v>26</v>
+      </c>
+      <c r="E11">
+        <v>74</v>
+      </c>
+      <c r="G11">
+        <v>51</v>
+      </c>
+      <c r="H11">
+        <v>49</v>
+      </c>
+      <c r="I11">
+        <v>21</v>
+      </c>
+      <c r="J11">
+        <v>79</v>
+      </c>
+      <c r="L11">
+        <v>91</v>
+      </c>
+      <c r="M11">
+        <v>9</v>
+      </c>
+      <c r="N11">
+        <v>11</v>
+      </c>
+      <c r="O11">
+        <v>89</v>
+      </c>
+      <c r="Q11">
+        <f t="shared" si="6"/>
+        <v>36.5</v>
+      </c>
+      <c r="R11">
+        <f t="shared" si="7"/>
+        <v>35</v>
+      </c>
+      <c r="S11">
+        <f t="shared" si="8"/>
+        <v>10</v>
+      </c>
+      <c r="T11">
+        <f t="shared" si="9"/>
+        <v>27.166666666666668</v>
+      </c>
+      <c r="U11">
+        <f t="shared" si="10"/>
+        <v>10</v>
+      </c>
+      <c r="V11">
+        <f t="shared" si="11"/>
+        <v>17.166666666666668</v>
       </c>
     </row>
   </sheetData>
@@ -14878,7 +15727,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEC9CF4A-6F3D-4BA0-B506-17E3C93FB04B}">
-  <dimension ref="A2:AF9"/>
+  <dimension ref="A2:AF14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="2" spans="1:32" x14ac:dyDescent="0.3">
@@ -15360,6 +16209,232 @@
         <v>11.833333333333332</v>
       </c>
     </row>
+    <row r="12" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B12">
+        <v>69</v>
+      </c>
+      <c r="C12">
+        <v>31</v>
+      </c>
+      <c r="D12">
+        <v>11</v>
+      </c>
+      <c r="E12">
+        <v>89</v>
+      </c>
+      <c r="G12">
+        <v>80</v>
+      </c>
+      <c r="H12">
+        <v>20</v>
+      </c>
+      <c r="I12">
+        <v>22</v>
+      </c>
+      <c r="J12">
+        <v>78</v>
+      </c>
+      <c r="L12">
+        <v>89</v>
+      </c>
+      <c r="M12">
+        <v>11</v>
+      </c>
+      <c r="N12">
+        <v>16</v>
+      </c>
+      <c r="O12">
+        <v>84</v>
+      </c>
+      <c r="Q12">
+        <f t="shared" ref="Q10:Q14" si="6">AVERAGE(C12,D12)</f>
+        <v>21</v>
+      </c>
+      <c r="R12">
+        <f t="shared" ref="R10:R14" si="7">AVERAGE(H12,I12)</f>
+        <v>21</v>
+      </c>
+      <c r="S12">
+        <f t="shared" ref="S10:S14" si="8">AVERAGE(M12,N12)</f>
+        <v>13.5</v>
+      </c>
+      <c r="T12">
+        <f t="shared" ref="T10:T14" si="9">AVERAGE(Q12:S12)</f>
+        <v>18.5</v>
+      </c>
+      <c r="U12">
+        <f>AVERAGE(Q12:Q17)</f>
+        <v>22.333333333333332</v>
+      </c>
+      <c r="V12">
+        <f>_xlfn.STDEV.S(Q12:Q17)</f>
+        <v>3.2145502536643242</v>
+      </c>
+      <c r="W12">
+        <f>AVERAGE(R12:R17)</f>
+        <v>21</v>
+      </c>
+      <c r="X12">
+        <f>_xlfn.STDEV.S(R12:R17)</f>
+        <v>4</v>
+      </c>
+      <c r="Y12">
+        <f>AVERAGE(S12:S18)</f>
+        <v>10.333333333333334</v>
+      </c>
+      <c r="Z12">
+        <f>_xlfn.STDEV.S(S12:S17)</f>
+        <v>3.2532035493238571</v>
+      </c>
+      <c r="AA12">
+        <f>AVERAGE(T12:T17)</f>
+        <v>17.888888888888889</v>
+      </c>
+      <c r="AB12">
+        <f>_xlfn.STDEV.S(T12:T17)</f>
+        <v>1.0584754935143132</v>
+      </c>
+      <c r="AC12">
+        <f t="shared" ref="AC10:AC14" si="10">MIN(Q12:S12)</f>
+        <v>13.5</v>
+      </c>
+      <c r="AD12">
+        <f t="shared" ref="AD10:AD14" si="11">T12-AC12</f>
+        <v>5</v>
+      </c>
+      <c r="AE12">
+        <f>AVERAGE(AD12:AD17)</f>
+        <v>7.5555555555555562</v>
+      </c>
+      <c r="AF12">
+        <f>_xlfn.STDEV.S(AD12:AD17)</f>
+        <v>2.364866294865863</v>
+      </c>
+    </row>
+    <row r="13" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B13">
+        <v>75</v>
+      </c>
+      <c r="C13">
+        <v>25</v>
+      </c>
+      <c r="D13">
+        <v>15</v>
+      </c>
+      <c r="E13">
+        <v>85</v>
+      </c>
+      <c r="G13">
+        <v>86</v>
+      </c>
+      <c r="H13">
+        <v>14</v>
+      </c>
+      <c r="I13">
+        <v>36</v>
+      </c>
+      <c r="J13">
+        <v>64</v>
+      </c>
+      <c r="L13">
+        <v>92</v>
+      </c>
+      <c r="M13">
+        <v>8</v>
+      </c>
+      <c r="N13">
+        <v>13</v>
+      </c>
+      <c r="O13">
+        <v>87</v>
+      </c>
+      <c r="Q13">
+        <f t="shared" si="6"/>
+        <v>20</v>
+      </c>
+      <c r="R13">
+        <f t="shared" si="7"/>
+        <v>25</v>
+      </c>
+      <c r="S13">
+        <f t="shared" si="8"/>
+        <v>10.5</v>
+      </c>
+      <c r="T13">
+        <f t="shared" si="9"/>
+        <v>18.5</v>
+      </c>
+      <c r="AC13">
+        <f t="shared" si="10"/>
+        <v>10.5</v>
+      </c>
+      <c r="AD13">
+        <f t="shared" si="11"/>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B14">
+        <v>62</v>
+      </c>
+      <c r="C14">
+        <v>38</v>
+      </c>
+      <c r="D14">
+        <v>14</v>
+      </c>
+      <c r="E14">
+        <v>86</v>
+      </c>
+      <c r="G14">
+        <v>84</v>
+      </c>
+      <c r="H14">
+        <v>16</v>
+      </c>
+      <c r="I14">
+        <v>18</v>
+      </c>
+      <c r="J14">
+        <v>82</v>
+      </c>
+      <c r="L14">
+        <v>94</v>
+      </c>
+      <c r="M14">
+        <v>6</v>
+      </c>
+      <c r="N14">
+        <v>8</v>
+      </c>
+      <c r="O14">
+        <v>92</v>
+      </c>
+      <c r="Q14">
+        <f t="shared" si="6"/>
+        <v>26</v>
+      </c>
+      <c r="R14">
+        <f t="shared" si="7"/>
+        <v>17</v>
+      </c>
+      <c r="S14">
+        <f t="shared" si="8"/>
+        <v>7</v>
+      </c>
+      <c r="T14">
+        <f t="shared" si="9"/>
+        <v>16.666666666666668</v>
+      </c>
+      <c r="AC14">
+        <f t="shared" si="10"/>
+        <v>7</v>
+      </c>
+      <c r="AD14">
+        <f t="shared" si="11"/>
+        <v>9.6666666666666679</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>